<commit_message>
Data for indicator Value of energy
</commit_message>
<xml_diff>
--- a/import/raw_data/id_parameter.xlsx
+++ b/import/raw_data/id_parameter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ren\Documents\GitHub\micat\import\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FE9922-70A4-4F14-B5CD-B5632C01553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E6483E-AEAE-4B03-A2F8-4E7F9FFA8E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52095" yWindow="2415" windowWidth="30555" windowHeight="17865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32205" yWindow="-4515" windowWidth="17610" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="161">
   <si>
     <t>id</t>
   </si>
@@ -489,6 +489,36 @@
   </si>
   <si>
     <t>Total energy system costs including balancing, profile, and grid costs, associated with integrating VRE at different penetration levels. [€/MWh]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wholesale price </t>
+  </si>
+  <si>
+    <t>Wholesale price of primary energy carrier (€/ktoe)</t>
+  </si>
+  <si>
+    <t>ETS price</t>
+  </si>
+  <si>
+    <t>ETS price per primary energy carrier (€/ktoe)</t>
+  </si>
+  <si>
+    <t>VNFC_el</t>
+  </si>
+  <si>
+    <t>VNFC_heat</t>
+  </si>
+  <si>
+    <t>Variable non fuel cost (electricity production) (€/ktoe)</t>
+  </si>
+  <si>
+    <t>Variable non fuel cost (heat production) (€/ktoe)</t>
+  </si>
+  <si>
+    <t>Value of energy</t>
+  </si>
+  <si>
+    <t>Value of energy which was produced by RES</t>
   </si>
 </sst>
 </file>
@@ -825,7 +855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.453125" customWidth="1"/>
@@ -1680,6 +1710,61 @@
         <v>150</v>
       </c>
     </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>151</v>
+      </c>
+      <c r="C78" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>153</v>
+      </c>
+      <c r="C79" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>155</v>
+      </c>
+      <c r="C80" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>156</v>
+      </c>
+      <c r="C81" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>159</v>
+      </c>
+      <c r="C82" t="s">
+        <v>160</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1687,27 +1772,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="89bcd336-abeb-4a08-b6b9-8f1906e00f8a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca47701c-f272-4f81-9665-1c7dbebc0776">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Type xmlns="ca47701c-f272-4f81-9665-1c7dbebc0776">id_table</Type>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010081027A5C4AB68A40A5017F28CDCC410C" ma:contentTypeVersion="17" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="f1f428d4bdb6f67b400b210b48125618">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca47701c-f272-4f81-9665-1c7dbebc0776" xmlns:ns3="89bcd336-abeb-4a08-b6b9-8f1906e00f8a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8189f6f0f7c839d9d0d3622fd62ec189" ns2:_="" ns3:_="">
     <xsd:import namespace="ca47701c-f272-4f81-9665-1c7dbebc0776"/>
@@ -1960,10 +2024,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="89bcd336-abeb-4a08-b6b9-8f1906e00f8a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca47701c-f272-4f81-9665-1c7dbebc0776">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Type xmlns="ca47701c-f272-4f81-9665-1c7dbebc0776">id_table</Type>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8500D24-9B3E-4E37-8AAD-EB7D9C788023}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABFDCFC1-0950-4DFE-9D9B-4AF680B2B273}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca47701c-f272-4f81-9665-1c7dbebc0776"/>
+    <ds:schemaRef ds:uri="89bcd336-abeb-4a08-b6b9-8f1906e00f8a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1980,20 +2076,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABFDCFC1-0950-4DFE-9D9B-4AF680B2B273}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8500D24-9B3E-4E37-8AAD-EB7D9C788023}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca47701c-f272-4f81-9665-1c7dbebc0776"/>
-    <ds:schemaRef ds:uri="89bcd336-abeb-4a08-b6b9-8f1906e00f8a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>